<commit_message>
patched "2307" name bugs to "Z307"
</commit_message>
<xml_diff>
--- a/supplemental/csi_surface_roughness/csi_surface_roughness_summary.xlsx
+++ b/supplemental/csi_surface_roughness/csi_surface_roughness_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jakep\Documents\Optics_local\UofA\bsdf-tools\supplemental\csi_surface_roughness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B285842-ED3A-48C3-8E80-124961217A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D0A130-C5F0-4E57-8BC4-E93001AC173A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3468" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
     <t>DEEP SPACE BLACK - Full Spectrum Basic</t>
   </si>
   <si>
-    <t>Aeroglaze 9924 Primer with Aeroglaze 2307 Black</t>
-  </si>
-  <si>
     <t>Vacuum Black on Aluminum</t>
   </si>
   <si>
@@ -162,6 +159,9 @@
   </si>
   <si>
     <t>**tried various CSI settings, but none could register a measurement.</t>
+  </si>
+  <si>
+    <t>Aeroglaze 9924 Primer with Aeroglaze Z307 Black</t>
   </si>
 </sst>
 </file>
@@ -790,12 +790,12 @@
     </row>
     <row r="2" spans="2:33" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="R2" s="19"/>
       <c r="S2" s="10"/>
       <c r="T2" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AG2" s="19"/>
     </row>
@@ -804,17 +804,17 @@
       <c r="C3" s="10"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="O3" s="10" t="s">
-        <v>35</v>
       </c>
       <c r="R3" s="19"/>
       <c r="T3" s="34" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U3" s="35"/>
       <c r="V3" s="35"/>
@@ -822,7 +822,7 @@
       <c r="X3" s="35"/>
       <c r="Y3" s="36"/>
       <c r="Z3" s="34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AA3" s="35"/>
       <c r="AB3" s="35"/>
@@ -833,86 +833,86 @@
     </row>
     <row r="4" spans="2:33" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N4" s="10"/>
       <c r="O4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q4" s="10"/>
       <c r="R4" s="19"/>
       <c r="T4" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="U4" s="17" t="s">
+      <c r="V4" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="V4" s="17" t="s">
+      <c r="W4" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="W4" s="17" t="s">
+      <c r="X4" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="X4" s="17" t="s">
+      <c r="Y4" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="Y4" s="18" t="s">
-        <v>30</v>
-      </c>
       <c r="Z4" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="17" t="s">
+      <c r="AB4" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="AB4" s="17" t="s">
+      <c r="AC4" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="AC4" s="17" t="s">
+      <c r="AD4" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="AD4" s="17" t="s">
+      <c r="AE4" s="18" t="s">
         <v>29</v>
-      </c>
-      <c r="AE4" s="18" t="s">
-        <v>30</v>
       </c>
       <c r="AG4" s="19"/>
     </row>
     <row r="5" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B5" s="25" t="s">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="C5" s="26">
         <v>46080</v>
@@ -931,16 +931,16 @@
         <v>20</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M5" s="30">
         <v>3</v>
@@ -984,7 +984,7 @@
     </row>
     <row r="6" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B6" s="21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" s="22">
         <v>46080</v>
@@ -1003,16 +1003,16 @@
         <v>20</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M6" s="31">
         <v>3</v>
@@ -1052,7 +1052,7 @@
     </row>
     <row r="7" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B7" s="21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="22">
         <v>46080</v>
@@ -1071,16 +1071,16 @@
         <v>20</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M7" s="31">
         <v>3</v>
@@ -1120,7 +1120,7 @@
     </row>
     <row r="8" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B8" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8" s="22">
         <v>46080</v>
@@ -1139,16 +1139,16 @@
         <v>40</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M8" s="31">
         <v>3</v>
@@ -1204,7 +1204,7 @@
     </row>
     <row r="9" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B9" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" s="22">
         <v>46080</v>
@@ -1223,16 +1223,16 @@
         <v>20</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M9" s="31">
         <v>3</v>
@@ -1295,16 +1295,16 @@
         <v>40</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M10" s="31">
         <v>3</v>
@@ -1344,7 +1344,7 @@
     </row>
     <row r="11" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B11" s="21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="22">
         <v>46080</v>
@@ -1363,16 +1363,16 @@
         <v>145</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M11" s="31">
         <v>3</v>
@@ -1412,7 +1412,7 @@
     </row>
     <row r="12" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C12" s="22">
         <v>45898</v>
@@ -1431,16 +1431,16 @@
         <v>20</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M12" s="31">
         <v>3</v>
@@ -1476,7 +1476,7 @@
     </row>
     <row r="13" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" s="22">
         <v>46080</v>
@@ -1495,16 +1495,16 @@
         <v>20</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M13" s="31">
         <v>3</v>
@@ -1544,49 +1544,49 @@
     </row>
     <row r="14" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" s="22">
         <v>46080</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G14" s="11"/>
       <c r="H14" s="28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M14" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N14" s="11"/>
       <c r="O14" s="28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P14" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q14" s="11"/>
       <c r="R14" s="20"/>
       <c r="S14" s="12"/>
       <c r="T14" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
@@ -1594,7 +1594,7 @@
       <c r="X14" s="1"/>
       <c r="Y14" s="7"/>
       <c r="Z14" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AA14" s="1"/>
       <c r="AB14" s="1"/>
@@ -1605,7 +1605,7 @@
     </row>
     <row r="15" spans="2:33" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="23" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C15" s="24">
         <v>46080</v>
@@ -1624,16 +1624,16 @@
         <v>10</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M15" s="32">
         <v>3</v>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N17" s="10"/>
       <c r="R17" s="19"/>
@@ -1702,7 +1702,7 @@
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>

</xml_diff>